<commit_message>
modified:   Planning/Week 27 - Itinerary 06.29.2026.xlsx
</commit_message>
<xml_diff>
--- a/Planning/Week 27 - Itinerary 06.29.2026.xlsx
+++ b/Planning/Week 27 - Itinerary 06.29.2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chris\Documents\GitHub\dex\Planning\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B127D58-E7EB-49FE-BA4A-1B104AB697D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D1CE150-6EA2-4AED-A869-5912D9EB0942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="61">
   <si>
     <t>Itinerary Week of:</t>
   </si>
@@ -194,129 +194,6 @@
     <t>FIN - FL4200 ($177K Active Project) - Glenn Spalding - (267) 492-1100 - Montgomeryville, PA - check project status, identify next opportunity</t>
   </si>
   <si>
-    <t>Thursday - Upper Bucks / Souderton</t>
-  </si>
-  <si>
-    <t>Klover Prefab</t>
-  </si>
-  <si>
-    <t>TrenchTech, Inc.</t>
-  </si>
-  <si>
-    <t>ALL - Plasma ($240K Quoting) + VEC - Robotic Welder ($100K Favorable) - (800) 443-6832 - Morrisville, PA - advance plasma quote, requalify robotics</t>
-  </si>
-  <si>
-    <t>Scaletron Industries Inc</t>
-  </si>
-  <si>
-    <t>MAG - FL6300RD ($250K Quoting) + TRU - TB3170/5170 ($249K Quoting) - Ed Dougherty, President - (215) 766-2670 - Plumsteadville, PA - advance both quotes</t>
-  </si>
-  <si>
-    <t>Bracalente Manufacturing</t>
-  </si>
-  <si>
-    <t>PMI - NC24 LS-Type ($78K Active Project) - Rich Nast, GM / Dave Borish, VP-COO - (215) 536-3077 - Telford, PA - check demo status</t>
-  </si>
-  <si>
-    <t>Vulcan Spring and Manufacturing</t>
-  </si>
-  <si>
-    <t>TRU - TLS7000 ($300K Active Project) - 2 months since last touch - check project milestones, identify upsell</t>
-  </si>
-  <si>
-    <t>J.I. Landis Welding</t>
-  </si>
-  <si>
-    <t>WIL Knee Mill ($13K) + CNC Lathe ($26K) + Manual Lathe ($45K) - Willis deals, confirm pricing and timeline</t>
-  </si>
-  <si>
-    <t>AW Mercer</t>
-  </si>
-  <si>
-    <t>FIN - FL6300RDDR ($355K Quoting) + MAM AutoTend ($218K Discovery) + HAE Pemserter ($25K Quoting) - advance deburring quote, qualify automation interest</t>
-  </si>
-  <si>
-    <t>Rise Construction Enterprises</t>
-  </si>
-  <si>
-    <t>PRO - PCR41 ($458K Quoting) - visit overdue since 7/25/25 - qualify interest, advance beam line opp</t>
-  </si>
-  <si>
-    <t>Szoke Brothers Inc (call)</t>
-  </si>
-  <si>
-    <t>ALL - Plasma ($228K Favorable) - Tom Szoke - (610) 760-0588 - overdue since 4/13, advance to quote</t>
-  </si>
-  <si>
-    <t>Friday - Office Day + Calls</t>
-  </si>
-  <si>
-    <t>Priority Calls (AM)</t>
-  </si>
-  <si>
-    <t>Call block 8:30-11:30 - light day before July 4 weekend. Include TRU N700 Nibbler follow-up.</t>
-  </si>
-  <si>
-    <t>Hadco Metal Trading Co (call)</t>
-  </si>
-  <si>
-    <t>TRU - TL3080/3060/3040 24kW ($1.42M Negotiation) + SOU N2 Gen ($295K) - Evgeny Voytovich - (215) 680-7239 - Bensalem - confirm closing timeline</t>
-  </si>
-  <si>
-    <t>Pennsylvania Steel Company (call)</t>
-  </si>
-  <si>
-    <t>PMI - T1 Plate Saw ($304K Quoting) + PMI HC230/NHC280 ($295K Discovery) - Mike Loveland - (215) 633-9600 - Bensalem - schedule in-person next week</t>
-  </si>
-  <si>
-    <t>Hanwha Philly Shipyard (call)</t>
-  </si>
-  <si>
-    <t>BAY Tandem ($5.26M Neg) + BAY Small ($1.09M Neg) + KAL ShotBlast ($3.6M) - $10.9M pipeline, last touch 5/11 - (215) 875-2600 - schedule formal site meeting</t>
-  </si>
-  <si>
-    <t>Pocono Metals (call)</t>
-  </si>
-  <si>
-    <t>Used EMI - follow up, confirm decision timeline - P1 overdue</t>
-  </si>
-  <si>
-    <t>Rybnick Mechanical (call)</t>
-  </si>
-  <si>
-    <t>FLO - Waterjet ($165K Active) + USE-GEKA Hydracrop ($26K Quoting) - schedule in-person meeting, bring Eric Marciniak from Flow</t>
-  </si>
-  <si>
-    <t>EVS Metal - East Stroudsburg (call)</t>
-  </si>
-  <si>
-    <t>MAG - Finishline ($190K Active) + MAM AutoTend ($218K Discovery) - East Stroudsburg, PA - check Finishline status, advance MAM</t>
-  </si>
-  <si>
-    <t>SMF Truck Equipment (call)</t>
-  </si>
-  <si>
-    <t>ALL - Plasma ($298K Quoting) - David Dunker - (610) 824-7000 - Palmerton, PA - advance quote</t>
-  </si>
-  <si>
-    <t>Prompton Tool (call)</t>
-  </si>
-  <si>
-    <t>TRU - MRC 7050/New 7036 ($165K Quoting) - (570) 253-4141 - Honesdale, PA - advance quote to close</t>
-  </si>
-  <si>
-    <t>Weekly Strategy Session (1:00-2:30)</t>
-  </si>
-  <si>
-    <t>Pipeline review, update opp files Mon-Thu, build Week 28 routes. Q3 started July 1 - set Q3 goals.</t>
-  </si>
-  <si>
-    <t>Follow-Ups &amp; Admin (2:30-4:00)</t>
-  </si>
-  <si>
-    <t>Post-visit emails, update SF activities, Q3 goal-setting.</t>
-  </si>
-  <si>
     <t>TRU - TL3030 Laser ($755K Quoting) - Ron DePack, Operations Manager/GM - (610) 821-0210 - Nazareth, PA - qualify timeline and champion</t>
   </si>
   <si>
@@ -332,7 +209,13 @@
     <t>VIR - LTG ($43K Favorable) + EMI - ELSQRD/TPC24 ($147K Quoting) - 3+ weeks since last touch - close Virtek, advance EMI</t>
   </si>
   <si>
-    <t>ALL - Plasma ($252K Quoting) + TRU Laser + BAY Brake + HEM Saw (multi-opp site) - (215) 536-7706 - Quakertown, PA - ask Ian for priorities</t>
+    <t>Holiday</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>Friday</t>
   </si>
 </sst>
 </file>
@@ -459,9 +342,34 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -469,37 +377,12 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="14" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -768,7 +651,7 @@
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" style="23" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" style="18" customWidth="1"/>
     <col min="3" max="3" width="75" style="8" customWidth="1"/>
   </cols>
   <sheetData>
@@ -785,23 +668,23 @@
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="11"/>
+      <c r="C2" s="20"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="11"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="20"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="16" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -810,498 +693,422 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="6"/>
-      <c r="B5" s="21"/>
+      <c r="B5" s="17"/>
       <c r="C5" s="6"/>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="14">
+      <c r="B6" s="10">
         <f>B1</f>
         <v>46202</v>
       </c>
-      <c r="C6" s="13"/>
+      <c r="C6" s="9"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="18"/>
-      <c r="C7" s="15" t="s">
+      <c r="B7" s="14"/>
+      <c r="C7" s="11" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="17"/>
-      <c r="C8" s="16" t="s">
+      <c r="B8" s="13"/>
+      <c r="C8" s="12" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="17"/>
-      <c r="C9" s="19" t="s">
-        <v>94</v>
+      <c r="B9" s="13"/>
+      <c r="C9" s="15" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="17"/>
-      <c r="C10" s="16" t="s">
+      <c r="B10" s="13"/>
+      <c r="C10" s="12" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="17"/>
-      <c r="C11" s="16" t="s">
+      <c r="B11" s="13"/>
+      <c r="C11" s="12" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="17"/>
-      <c r="C12" s="16" t="s">
+      <c r="B12" s="13"/>
+      <c r="C12" s="12" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="17"/>
-      <c r="C13" s="19" t="s">
-        <v>95</v>
+      <c r="B13" s="13"/>
+      <c r="C13" s="15" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="17"/>
-      <c r="C14" s="16" t="s">
+      <c r="B14" s="13"/>
+      <c r="C14" s="12" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="14">
+      <c r="B15" s="10">
         <f>B1+1</f>
         <v>46203</v>
       </c>
-      <c r="C15" s="13"/>
+      <c r="C15" s="9"/>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="17"/>
-      <c r="C16" s="16" t="s">
+      <c r="B16" s="13"/>
+      <c r="C16" s="12" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="17"/>
-      <c r="C17" s="16" t="s">
+      <c r="B17" s="13"/>
+      <c r="C17" s="12" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="16" t="s">
+      <c r="A18" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="16" t="s">
+      <c r="B18" s="13"/>
+      <c r="C18" s="12" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="16" t="s">
+      <c r="A19" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="17"/>
-      <c r="C19" s="16" t="s">
+      <c r="B19" s="13"/>
+      <c r="C19" s="12" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="16" t="s">
+      <c r="A20" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="17"/>
-      <c r="C20" s="16" t="s">
+      <c r="B20" s="13"/>
+      <c r="C20" s="12" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="16" t="s">
+      <c r="A21" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="17"/>
-      <c r="C21" s="16" t="s">
+      <c r="B21" s="13"/>
+      <c r="C21" s="12" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="16" t="s">
+      <c r="A22" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="17"/>
-      <c r="C22" s="16" t="s">
+      <c r="B22" s="13"/>
+      <c r="C22" s="12" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="13" t="s">
+      <c r="A23" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B23" s="14">
+      <c r="B23" s="10">
         <f>B1+2</f>
         <v>46204</v>
       </c>
-      <c r="C23" s="13"/>
+      <c r="C23" s="9"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="16" t="s">
+      <c r="A24" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B24" s="17"/>
-      <c r="C24" s="19" t="s">
-        <v>96</v>
+      <c r="B24" s="13"/>
+      <c r="C24" s="15" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="16" t="s">
+      <c r="B25" s="13"/>
+      <c r="C25" s="12" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="16" t="s">
+      <c r="A26" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="B26" s="17"/>
-      <c r="C26" s="16" t="s">
+      <c r="B26" s="13"/>
+      <c r="C26" s="12" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="16" t="s">
+      <c r="A27" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="B27" s="17"/>
-      <c r="C27" s="16" t="s">
+      <c r="B27" s="13"/>
+      <c r="C27" s="12" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="16" t="s">
+      <c r="A28" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B28" s="17"/>
-      <c r="C28" s="19" t="s">
-        <v>97</v>
+      <c r="B28" s="13"/>
+      <c r="C28" s="15" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="16" t="s">
+      <c r="A29" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="B29" s="17"/>
-      <c r="C29" s="16" t="s">
+      <c r="B29" s="13"/>
+      <c r="C29" s="12" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="16" t="s">
+      <c r="A30" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B30" s="17"/>
-      <c r="C30" s="16" t="s">
+      <c r="B30" s="13"/>
+      <c r="C30" s="12" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="s">
+      <c r="A31" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B31" s="17"/>
-      <c r="C31" s="19" t="s">
-        <v>98</v>
+      <c r="B31" s="13"/>
+      <c r="C31" s="15" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="16" t="s">
+      <c r="A32" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="B32" s="17"/>
-      <c r="C32" s="16" t="s">
+      <c r="B32" s="13"/>
+      <c r="C32" s="12" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="B33" s="14">
+      <c r="A33" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="B33" s="10">
         <f>B1+3</f>
         <v>46205</v>
       </c>
-      <c r="C33" s="13"/>
+      <c r="C33" s="9"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="B34" s="17"/>
-      <c r="C34" s="19" t="s">
-        <v>99</v>
-      </c>
+      <c r="A34" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B34" s="14"/>
+      <c r="C34" s="11"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="B35" s="17"/>
-      <c r="C35" s="16" t="s">
-        <v>56</v>
-      </c>
+      <c r="A35" s="11"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="11"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="B36" s="17"/>
-      <c r="C36" s="16" t="s">
-        <v>58</v>
-      </c>
+      <c r="A36" s="11"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="11"/>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="B37" s="17"/>
-      <c r="C37" s="16" t="s">
+      <c r="A37" s="11"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="11"/>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="11"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="11"/>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="11"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="11"/>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="11"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="11"/>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="11"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="11"/>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="11"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="11"/>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="23" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="B38" s="17"/>
-      <c r="C38" s="16" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="B39" s="18"/>
-      <c r="C39" s="15" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="B40" s="17"/>
-      <c r="C40" s="16" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="B41" s="18"/>
-      <c r="C41" s="15" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="16" t="s">
-        <v>69</v>
-      </c>
-      <c r="B42" s="17"/>
-      <c r="C42" s="16" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="B43" s="14">
+      <c r="B43" s="10">
         <f>B1+4</f>
         <v>46206</v>
       </c>
-      <c r="C43" s="13"/>
+      <c r="C43" s="9"/>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="B44" s="18"/>
-      <c r="C44" s="15" t="s">
-        <v>73</v>
-      </c>
+      <c r="A44" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B44" s="14"/>
+      <c r="C44" s="11"/>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="B45" s="17"/>
-      <c r="C45" s="16" t="s">
-        <v>75</v>
-      </c>
+      <c r="A45" s="11"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="11"/>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="16" t="s">
-        <v>76</v>
-      </c>
-      <c r="B46" s="17"/>
-      <c r="C46" s="16" t="s">
-        <v>77</v>
-      </c>
+      <c r="A46" s="11"/>
+      <c r="B46" s="14"/>
+      <c r="C46" s="11"/>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" s="16" t="s">
-        <v>78</v>
-      </c>
-      <c r="B47" s="17"/>
-      <c r="C47" s="16" t="s">
-        <v>79</v>
-      </c>
+      <c r="A47" s="11"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="11"/>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="B48" s="17"/>
-      <c r="C48" s="16" t="s">
-        <v>81</v>
-      </c>
+      <c r="A48" s="11"/>
+      <c r="B48" s="14"/>
+      <c r="C48" s="11"/>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="B49" s="17"/>
-      <c r="C49" s="16" t="s">
-        <v>83</v>
-      </c>
+      <c r="A49" s="11"/>
+      <c r="B49" s="14"/>
+      <c r="C49" s="11"/>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="16" t="s">
-        <v>84</v>
-      </c>
-      <c r="B50" s="17"/>
-      <c r="C50" s="16" t="s">
-        <v>85</v>
-      </c>
+      <c r="A50" s="11"/>
+      <c r="B50" s="14"/>
+      <c r="C50" s="11"/>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="16" t="s">
-        <v>86</v>
-      </c>
-      <c r="B51" s="17"/>
-      <c r="C51" s="16" t="s">
-        <v>87</v>
-      </c>
+      <c r="A51" s="11"/>
+      <c r="B51" s="14"/>
+      <c r="C51" s="11"/>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="B52" s="17"/>
-      <c r="C52" s="16" t="s">
-        <v>89</v>
-      </c>
+      <c r="A52" s="11"/>
+      <c r="B52" s="14"/>
+      <c r="C52" s="11"/>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="15" t="s">
-        <v>90</v>
-      </c>
-      <c r="B53" s="18"/>
-      <c r="C53" s="15" t="s">
-        <v>91</v>
-      </c>
+      <c r="A53" s="11"/>
+      <c r="B53" s="14"/>
+      <c r="C53" s="11"/>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="B54" s="18"/>
-      <c r="C54" s="15" t="s">
-        <v>93</v>
-      </c>
+      <c r="A54" s="11"/>
+      <c r="B54" s="14"/>
+      <c r="C54" s="11"/>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="9"/>
-      <c r="B55" s="22"/>
-      <c r="C55" s="9"/>
+      <c r="A55" s="11"/>
+      <c r="B55" s="14"/>
+      <c r="C55" s="11"/>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="9"/>
-      <c r="B56" s="22"/>
-      <c r="C56" s="9"/>
+      <c r="A56" s="11"/>
+      <c r="B56" s="14"/>
+      <c r="C56" s="11"/>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="6"/>
-      <c r="B57" s="21"/>
-      <c r="C57" s="6"/>
+      <c r="A57" s="11"/>
+      <c r="B57" s="14"/>
+      <c r="C57" s="11"/>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="6"/>
-      <c r="B58" s="21"/>
+      <c r="B58" s="17"/>
       <c r="C58" s="6"/>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="6"/>
-      <c r="B59" s="21"/>
+      <c r="B59" s="17"/>
       <c r="C59" s="6"/>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="6"/>
-      <c r="B60" s="21"/>
+      <c r="B60" s="17"/>
       <c r="C60" s="6"/>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="6"/>
-      <c r="B61" s="21"/>
+      <c r="B61" s="17"/>
       <c r="C61" s="6"/>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="6"/>
-      <c r="B62" s="21"/>
+      <c r="B62" s="17"/>
       <c r="C62" s="6"/>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="6"/>
-      <c r="B63" s="21"/>
+      <c r="B63" s="17"/>
       <c r="C63" s="6"/>
     </row>
   </sheetData>

</xml_diff>